<commit_message>
Adding model comparison spreadsheet
</commit_message>
<xml_diff>
--- a/specifications/models_comparison.xlsx
+++ b/specifications/models_comparison.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\bcaetani\mestrado\object_orientation_extracted_features\specifications\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{625D7563-875A-46DC-B674-E418E5B70037}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E223C1C-5BB9-40EC-BA67-0A64EB6F1FF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="15264" yWindow="0" windowWidth="15552" windowHeight="16656" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,19 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
-  <si>
-    <t>Média do Erro Geodésico (Treinamento)</t>
-  </si>
-  <si>
-    <t>Média do Erro Geodésico (Teste)</t>
-  </si>
-  <si>
-    <t>RMSE do Erro Geodésico (Treinamento)</t>
-  </si>
-  <si>
-    <t>RMSE do Erro Geodésico (Teste)</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="39">
   <si>
     <t>Regressão Linear</t>
   </si>
@@ -54,10 +42,106 @@
     <t>SVM (Polinomial)</t>
   </si>
   <si>
-    <t>Tolerância mínima para 60% de acerto (Teste)</t>
-  </si>
-  <si>
-    <t>Tolerância mínima para 80% de acerto (Teste)</t>
+    <t>37,4</t>
+  </si>
+  <si>
+    <t>38,8</t>
+  </si>
+  <si>
+    <t>49,4</t>
+  </si>
+  <si>
+    <t>---</t>
+  </si>
+  <si>
+    <t>2,3</t>
+  </si>
+  <si>
+    <t>2,4</t>
+  </si>
+  <si>
+    <t>2,6</t>
+  </si>
+  <si>
+    <t>Média do Erro Geodésico (Treinamento) [graus]</t>
+  </si>
+  <si>
+    <t>Média do Erro Geodésico (Teste) [graus]</t>
+  </si>
+  <si>
+    <t>RMSE do Erro Geodésico (Treinamento) [graus]</t>
+  </si>
+  <si>
+    <t>RMSE do Erro Geodésico (Teste) [graus]</t>
+  </si>
+  <si>
+    <t>Tolerância mínima para 60% de acerto (Teste) [graus]</t>
+  </si>
+  <si>
+    <t>Tolerância mínima para 80% de acerto (Teste) [graus]</t>
+  </si>
+  <si>
+    <t>9,6</t>
+  </si>
+  <si>
+    <t>17,6</t>
+  </si>
+  <si>
+    <t>7,4</t>
+  </si>
+  <si>
+    <t>3,3</t>
+  </si>
+  <si>
+    <t>7,0</t>
+  </si>
+  <si>
+    <t>11,8</t>
+  </si>
+  <si>
+    <t>5,5</t>
+  </si>
+  <si>
+    <t>2,2</t>
+  </si>
+  <si>
+    <t>9,4</t>
+  </si>
+  <si>
+    <t>5,3</t>
+  </si>
+  <si>
+    <t>8,9</t>
+  </si>
+  <si>
+    <t>4,5</t>
+  </si>
+  <si>
+    <t>6,1</t>
+  </si>
+  <si>
+    <t>9,1</t>
+  </si>
+  <si>
+    <t>5,2</t>
+  </si>
+  <si>
+    <t>Tolerância mínima para 60% de acerto (Treinamento) [graus]</t>
+  </si>
+  <si>
+    <t>Tolerância mínima para 80% de acerto (Treinamento) [graus]</t>
+  </si>
+  <si>
+    <t>2,5</t>
+  </si>
+  <si>
+    <t>3,1</t>
+  </si>
+  <si>
+    <t>&lt;1</t>
+  </si>
+  <si>
+    <t>1,5</t>
   </si>
 </sst>
 </file>
@@ -93,8 +177,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -375,10 +465,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="39" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="51.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.88671875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.88671875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.5546875" bestFit="1" customWidth="1"/>
@@ -388,49 +478,179 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s">
         <v>4</v>
-      </c>
-      <c r="C1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1" t="s">
-        <v>7</v>
-      </c>
-      <c r="F1" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>0</v>
+        <v>12</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>1</v>
+        <v>13</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>2</v>
+        <v>14</v>
+      </c>
+      <c r="B4" s="1">
+        <v>47.9</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>15</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>33</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" s="1">
+        <v>2</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>16</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="1">
+        <v>3</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" s="1">
+        <v>11</v>
+      </c>
+      <c r="D9" s="1">
+        <v>9</v>
+      </c>
+      <c r="E9" s="1">
+        <v>7</v>
+      </c>
+      <c r="F9" s="1">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>